<commit_message>
Regenerate sheets for the live URL and record live verification
Sheets now point at https://anishonly121.github.io/northwind-stays.
VERIFY_REPORT.md includes a run of every row against the live site in
Microsoft Edge.
</commit_message>
<xml_diff>
--- a/sheets/Northwind_NewFeature_Rows_1.1.0.xlsx
+++ b/sheets/Northwind_NewFeature_Rows_1.1.0.xlsx
@@ -1017,10 +1017,10 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1">
+    <row r="24" ht="45" customHeight="1">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>Rows that test login or the one-time code use the real login. All other rows start on a signed-in page with ?as=tester in the URL. That is a test shortcut that signs in tester@northwind.test straight away.</t>
+          <t>Rows that test login or the one-time code use the real login, and the Access control row starts signed out on purpose. All other rows start on a signed-in page with ?as=tester in the URL. That is a test shortcut that signs in tester@northwind.test straight away.</t>
         </is>
       </c>
     </row>

</xml_diff>